<commit_message>
Update national IDs spreadsheet in database directory
- Replaced the existing national IDs spreadsheet with an updated version in the database directory, ensuring consistency with the file path used in the UpsertEmployeesFromNationalIdsCommand.
- This change supports improved file management and aligns with recent refactoring efforts to streamline employee upsertion processes.
</commit_message>
<xml_diff>
--- a/database/data/national-ids.xlsx
+++ b/database/data/national-ids.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="120" windowWidth="18960" windowHeight="11760"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
-    <sheet name="ورقة2" sheetId="2" r:id="rId2"/>
-    <sheet name="ورقة3" sheetId="3" r:id="rId3"/>
+    <sheet name="ورقة1" sheetId="1" r:id="rId4"/>
+    <sheet name="ورقة2" sheetId="2" r:id="rId5"/>
+    <sheet name="ورقة3" sheetId="3" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
   <si>
     <t>نصيب عبدالرؤوف ابراهيم الصغير لاغه</t>
   </si>
@@ -57,6 +58,9 @@
     <t>ليلى حماتة محمد ابة</t>
   </si>
   <si>
+    <t>رقم اداري</t>
+  </si>
+  <si>
     <t>عبدالله محمد محمد مختار</t>
   </si>
   <si>
@@ -75,7 +79,7 @@
     <t>محمد عبدالغني علي اضويمر</t>
   </si>
   <si>
-    <t>عصام المبروك قشوط</t>
+    <t>عصام المبروك انطاط قشوط</t>
   </si>
   <si>
     <t>احمد ادريس فضل المهدي</t>
@@ -106,34 +110,44 @@
   </si>
   <si>
     <t>مولود احمد محمد الشيخ</t>
-  </si>
-  <si>
-    <t>رقم اداري</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
       <charset val="178"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="178"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="178"/>
     </font>
   </fonts>
   <fills count="2">
@@ -185,39 +199,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="1" numFmtId="1" fillId="0" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="1" numFmtId="1" fillId="0" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" readingOrder="2"/>
+    <xf xfId="0" fontId="2" numFmtId="1" fillId="0" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="سمة Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -500,16 +514,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="2" max="2" width="27.125" customWidth="1"/>
-    <col min="3" max="3" width="22.75" customWidth="1"/>
-    <col min="4" max="4" width="18.125" customWidth="1"/>
+    <col min="2" max="2" width="27.125" customWidth="true" style="0"/>
+    <col min="3" max="3" width="22.75" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18.125" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1">
+    <row r="1" spans="1:4" customHeight="1" ht="15.75">
       <c r="A1" s="3">
         <v>1532</v>
       </c>
@@ -521,7 +538,7 @@
       </c>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1">
+    <row r="2" spans="1:4" customHeight="1" ht="15.75">
       <c r="A2" s="4">
         <v>1642</v>
       </c>
@@ -533,7 +550,7 @@
       </c>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" ht="15.75" thickBot="1">
+    <row r="3" spans="1:4" customHeight="1" ht="15.75">
       <c r="A3" s="4">
         <v>1653</v>
       </c>
@@ -545,7 +562,7 @@
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="15.75" thickBot="1">
+    <row r="4" spans="1:4" customHeight="1" ht="15.75">
       <c r="A4" s="4">
         <v>1693</v>
       </c>
@@ -557,7 +574,7 @@
       </c>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1">
+    <row r="5" spans="1:4" customHeight="1" ht="15.75">
       <c r="A5" s="4">
         <v>2492</v>
       </c>
@@ -569,7 +586,7 @@
       </c>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" ht="15.75" thickBot="1">
+    <row r="6" spans="1:4" customHeight="1" ht="15.75">
       <c r="A6" s="4">
         <v>2763</v>
       </c>
@@ -581,7 +598,7 @@
       </c>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1">
+    <row r="7" spans="1:4" customHeight="1" ht="15.75">
       <c r="A7" s="4">
         <v>2885</v>
       </c>
@@ -593,7 +610,7 @@
       </c>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" ht="15.75" thickBot="1">
+    <row r="8" spans="1:4" customHeight="1" ht="15.75">
       <c r="A8" s="4">
         <v>4128</v>
       </c>
@@ -605,7 +622,7 @@
       </c>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1">
+    <row r="9" spans="1:4" customHeight="1" ht="15.75">
       <c r="A9" s="4">
         <v>5215</v>
       </c>
@@ -617,7 +634,7 @@
       </c>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="15.75" thickBot="1">
+    <row r="10" spans="1:4" customHeight="1" ht="15.75">
       <c r="A10" s="4">
         <v>5217</v>
       </c>
@@ -629,7 +646,7 @@
       </c>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1">
+    <row r="11" spans="1:4" customHeight="1" ht="15.75">
       <c r="A11" s="4">
         <v>7120</v>
       </c>
@@ -641,7 +658,7 @@
       </c>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" ht="15.75" thickBot="1">
+    <row r="12" spans="1:4" customHeight="1" ht="15.75">
       <c r="A12" s="4">
         <v>12037</v>
       </c>
@@ -651,7 +668,7 @@
       <c r="C12" s="5"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1">
+    <row r="13" spans="1:4" customHeight="1" ht="15.75">
       <c r="A13" s="4">
         <v>14027</v>
       </c>
@@ -662,215 +679,215 @@
         <v>6198603828</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" customHeight="1" ht="15.75">
       <c r="A14" s="4">
         <v>14033</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" s="5">
         <v>5198702828</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" customHeight="1" ht="15.75">
       <c r="A15" s="4">
         <v>14035</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C15" s="5">
         <v>5196805329</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" customHeight="1" ht="15.75">
       <c r="A16" s="4">
         <v>17010</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" s="5">
         <v>5197301641</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" customHeight="1" ht="15.75">
       <c r="A17" s="4">
         <v>17109</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17" s="5">
         <v>119910156249</v>
       </c>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" ht="15.75" thickBot="1">
+    <row r="18" spans="1:4" customHeight="1" ht="15.75">
       <c r="A18" s="4">
         <v>27013</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C18" s="7">
         <v>5196402769</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.75" thickBot="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" customHeight="1" ht="15.75">
       <c r="A19" s="4">
         <v>27068</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C19" s="7">
         <v>119880045493</v>
       </c>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" ht="15.75" thickBot="1">
+    <row r="20" spans="1:4" customHeight="1" ht="15.75">
       <c r="A20" s="4">
         <v>28104</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C20" s="7">
         <v>119750300015</v>
       </c>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" ht="15.75" thickBot="1">
+    <row r="21" spans="1:4" customHeight="1" ht="15.75">
       <c r="A21" s="4">
         <v>33092</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C21" s="7">
         <v>120010353384</v>
       </c>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" ht="15.75" thickBot="1">
+    <row r="22" spans="1:4" customHeight="1" ht="15.75">
       <c r="A22" s="4">
         <v>33106</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C22" s="7">
         <v>120030308210</v>
       </c>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" ht="15.75" thickBot="1">
+    <row r="23" spans="1:4" customHeight="1" ht="15.75">
       <c r="A23" s="4">
         <v>1731</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C23" s="5">
         <v>119740301738</v>
       </c>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="1:4" ht="15.75" thickBot="1">
+    <row r="24" spans="1:4" customHeight="1" ht="15.75">
       <c r="A24" s="4">
         <v>21026</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C24" s="5">
         <v>219960294848</v>
       </c>
       <c r="D24" s="4"/>
     </row>
-    <row r="25" spans="1:4" ht="15.75" thickBot="1">
+    <row r="25" spans="1:4" customHeight="1" ht="15.75">
       <c r="A25" s="4">
         <v>3019</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C25" s="5">
         <v>119630089704</v>
       </c>
       <c r="D25" s="4"/>
     </row>
-    <row r="26" spans="1:4" ht="15.75" thickBot="1">
+    <row r="26" spans="1:4" customHeight="1" ht="15.75">
       <c r="A26" s="4">
         <v>32032</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C26" s="5">
         <v>219990213970</v>
       </c>
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="1:4" ht="15.75" thickBot="1">
+    <row r="27" spans="1:4" customHeight="1" ht="15.75">
       <c r="A27" s="4">
         <v>6252</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C27" s="5">
         <v>219890263624</v>
       </c>
       <c r="D27" s="4"/>
     </row>
-    <row r="28" spans="1:4" ht="15.75" thickBot="1">
+    <row r="28" spans="1:4" customHeight="1" ht="15.75">
       <c r="A28" s="4">
         <v>14055</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C28" s="5">
         <v>219990147837</v>
       </c>
       <c r="D28" s="4"/>
     </row>
-    <row r="29" spans="1:4" ht="15.75" thickBot="1">
+    <row r="29" spans="1:4" customHeight="1" ht="15.75">
       <c r="A29" s="4">
         <v>14050</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C29" s="5">
         <v>220000390989</v>
       </c>
       <c r="D29" s="4"/>
     </row>
-    <row r="30" spans="1:4" ht="15.75" thickBot="1">
+    <row r="30" spans="1:4" customHeight="1" ht="15.75">
       <c r="A30" s="4">
         <v>14036</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C30" s="5">
         <v>119900405241</v>
@@ -878,27 +895,36 @@
       <c r="D30" s="4"/>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" r:id="rId1ps"/>
 </worksheet>
 </file>
</xml_diff>